<commit_message>
Update dashboard logic, add interactive table title, fix 15% collocation calculation
</commit_message>
<xml_diff>
--- a/dv_data_pm25_2025.xlsx
+++ b/dv_data_pm25_2025.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nlambini\Desktop\Collocation Tracking Python\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B6F612C2-B90D-4543-9D39-A94C5CEC3A5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5164BE77-FEE7-48B1-AD14-63719DA9AD21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{04EE28B2-F154-4399-9206-2B56A7747D3D}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{04EE28B2-F154-4399-9206-2B56A7747D3D}"/>
   </bookViews>
   <sheets>
     <sheet name="DesignValues" sheetId="1" r:id="rId1"/>
     <sheet name="AgencyName" sheetId="2" r:id="rId2"/>
     <sheet name="IDDataBase" sheetId="3" r:id="rId3"/>
+    <sheet name="AgencyPQAO" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029" iterate="1" iterateDelta="1.0000000000000001E-5"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2848" uniqueCount="1782">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2896" uniqueCount="1789">
   <si>
     <t>AQS ID</t>
   </si>
@@ -5384,6 +5385,27 @@
   </si>
   <si>
     <t>Extraction Date</t>
+  </si>
+  <si>
+    <t>Agency</t>
+  </si>
+  <si>
+    <t>PQAO</t>
+  </si>
+  <si>
+    <t>BAAQMD</t>
+  </si>
+  <si>
+    <t>CARB</t>
+  </si>
+  <si>
+    <t>NPS</t>
+  </si>
+  <si>
+    <t>SDCAPCD</t>
+  </si>
+  <si>
+    <t>SCAQMD</t>
   </si>
 </sst>
 </file>
@@ -21945,4 +21967,210 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABB7423F-069D-4940-A66C-1F730789A39D}">
+  <dimension ref="A1:B24"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="47.36328125" customWidth="1"/>
+    <col min="2" max="2" width="20.08984375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>1782</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1783</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1784</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>128</v>
+      </c>
+      <c r="B3" t="s">
+        <v>1785</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>137</v>
+      </c>
+      <c r="B4" t="s">
+        <v>1785</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>202</v>
+      </c>
+      <c r="B5" t="s">
+        <v>1785</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>248</v>
+      </c>
+      <c r="B6" t="s">
+        <v>1785</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>266</v>
+      </c>
+      <c r="B7" t="s">
+        <v>1785</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>334</v>
+      </c>
+      <c r="B8" t="s">
+        <v>1785</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>409</v>
+      </c>
+      <c r="B9" t="s">
+        <v>1785</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>351</v>
+      </c>
+      <c r="B10" t="s">
+        <v>1785</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>164</v>
+      </c>
+      <c r="B11" t="s">
+        <v>1786</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>355</v>
+      </c>
+      <c r="B12" t="s">
+        <v>1785</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>367</v>
+      </c>
+      <c r="B13" t="s">
+        <v>1785</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>403</v>
+      </c>
+      <c r="B14" t="s">
+        <v>1785</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>432</v>
+      </c>
+      <c r="B15" t="s">
+        <v>1787</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>182</v>
+      </c>
+      <c r="B16" t="s">
+        <v>1785</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>461</v>
+      </c>
+      <c r="B17" t="s">
+        <v>1785</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>476</v>
+      </c>
+      <c r="B18" t="s">
+        <v>1785</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>505</v>
+      </c>
+      <c r="B19" t="s">
+        <v>1785</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>514</v>
+      </c>
+      <c r="B20" t="s">
+        <v>1785</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>272</v>
+      </c>
+      <c r="B21" t="s">
+        <v>1788</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>544</v>
+      </c>
+      <c r="B22" t="s">
+        <v>1785</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>557</v>
+      </c>
+      <c r="B23" t="s">
+        <v>1785</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>523</v>
+      </c>
+      <c r="B24" t="s">
+        <v>1785</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>